<commit_message>
Period range filter, type chip filtering, dashboard polish
- Period range selector (С/По dropdowns) next to campaign selector
- Period chips: click = single month, range highlight, collapse >6, Весь период reset
- All dashboard widgets respect period range (KPIs, charts, table, map)
- Type filter chips now show only types present in current campaign
- Remove Тепловая карта tab from map widget
- Fix orphaned screen cleanup on period re-upload

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/samples/byd_feb.xlsx
+++ b/docs/samples/byd_feb.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91576D7F-13DB-4388-87E7-6B805A45A62E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148C6973-E095-4E0C-8DEA-2A7B377967D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,7 +11,7 @@
     <sheet name="Медиаплан" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Медиаплан!$A$2:$V$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Медиаплан!$A$2:$V$74</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -598,7 +598,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
@@ -662,6 +662,8 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
@@ -1016,10 +1018,12 @@
     <col min="9" max="9" width="14" style="2" customWidth="1"/>
     <col min="10" max="10" width="16" style="2" customWidth="1"/>
     <col min="11" max="12" width="20" customWidth="1"/>
-    <col min="13" max="16" width="22" customWidth="1"/>
-    <col min="17" max="17" width="12" customWidth="1"/>
+    <col min="13" max="15" width="22" customWidth="1"/>
+    <col min="16" max="16" width="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="10" customWidth="1"/>
-    <col min="19" max="20" width="12" customWidth="1"/>
+    <col min="19" max="19" width="12" customWidth="1"/>
+    <col min="20" max="20" width="14" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="10" customWidth="1"/>
     <col min="22" max="22" width="11.7109375" customWidth="1"/>
   </cols>
@@ -1055,6 +1059,10 @@
       <c r="K1" t="s">
         <v>0</v>
       </c>
+      <c r="L1">
+        <f>K3*28</f>
+        <v>10976</v>
+      </c>
       <c r="M1" t="s">
         <v>0</v>
       </c>
@@ -6112,6 +6120,10 @@
       </c>
     </row>
     <row r="74" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="P74" s="27">
+        <f>SUM(P3:P73)</f>
+        <v>405303281.92704004</v>
+      </c>
       <c r="Q74" s="21"/>
       <c r="R74" s="21"/>
       <c r="S74" s="21"/>
@@ -6120,10 +6132,16 @@
       <c r="V74" s="21"/>
     </row>
     <row r="75" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="Q75" s="21"/>
+      <c r="Q75" s="28">
+        <f>SUBTOTAL(9,Q3:Q74)</f>
+        <v>19643180</v>
+      </c>
       <c r="R75" s="21"/>
       <c r="S75" s="21"/>
-      <c r="T75" s="21"/>
+      <c r="T75" s="28">
+        <f>SUBTOTAL(9,T3:T74)</f>
+        <v>17455490</v>
+      </c>
       <c r="U75" s="21"/>
       <c r="V75" s="21"/>
     </row>
@@ -12395,7 +12413,7 @@
   <protectedRanges>
     <protectedRange algorithmName="SHA-512" hashValue="20tZejZtY/ZGRcGLZm0ZbWfCu51ejQGMqdRYwv0b9rb/5Q/ejFDHQOXySZDQbnMuPhvZC4Bfbq/BWdBxp9Ls4w==" saltValue="Q+V8rXhHsE4u/j5xUQJeAg==" spinCount="100000" sqref="B27:B73" name="Диапазон1_9_1_1_1_1_1"/>
   </protectedRanges>
-  <autoFilter ref="A2:V73" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A2:V74" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="T1:U1"/>
     <mergeCell ref="Q1:S1"/>

</xml_diff>